<commit_message>
Add DBS6 audit review (run 20260924-981b2555); flag new-campaign raises in DBS4
Review of the Decolure Bamboo Sheets 6 Piece ranking run and its stored review,
with swaps judged on the inventory planner and the run's dated arrivals, the
Queen hero split limited to the campaigns the push raises, and each rank freeze
read on the daily crawl. In DBS4, raises on campaigns missing from the export
are now flagged rather than held, since Command Center shows them as new
launches.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECNUyLvUafHehET6NevFNz
</commit_message>
<xml_diff>
--- a/docs/reviews/DBS4_Review_Rows_20260924-5e8a0f10.xlsx
+++ b/docs/reviews/DBS4_Review_Rows_20260924-5e8a0f10.xlsx
@@ -1561,13 +1561,13 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P13" t="n">
         <v>1.22</v>
       </c>
       <c r="Q13" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14">
@@ -1640,13 +1640,13 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P14" t="n">
         <v>1.22</v>
       </c>
       <c r="Q14" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15">
@@ -1719,13 +1719,13 @@
         </is>
       </c>
       <c r="O15" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P15" t="n">
         <v>1.22</v>
       </c>
       <c r="Q15" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16">
@@ -3457,13 +3457,13 @@
         </is>
       </c>
       <c r="O37" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P37" t="n">
         <v>1.22</v>
       </c>
       <c r="Q37" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="38">
@@ -3536,13 +3536,13 @@
         </is>
       </c>
       <c r="O38" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P38" t="n">
         <v>1.22</v>
       </c>
       <c r="Q38" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="39">
@@ -3615,13 +3615,13 @@
         </is>
       </c>
       <c r="O39" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P39" t="n">
         <v>1.22</v>
       </c>
       <c r="Q39" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="40">
@@ -4405,13 +4405,13 @@
         </is>
       </c>
       <c r="O49" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P49" t="n">
         <v>1.22</v>
       </c>
       <c r="Q49" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="50">
@@ -4484,13 +4484,13 @@
         </is>
       </c>
       <c r="O50" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P50" t="n">
         <v>1.22</v>
       </c>
       <c r="Q50" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="51">
@@ -5195,13 +5195,13 @@
         </is>
       </c>
       <c r="O59" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P59" t="n">
         <v>1.22</v>
       </c>
       <c r="Q59" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="60">
@@ -9330,12 +9330,12 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>deploy</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -9345,7 +9345,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>A raise on a campaign the export does not carry: no status, child, or read to check it against. Confirm the campaign and its child first.</t>
+          <t>A raise on a campaign the export’s campaign list does not carry, so no reviewer can recompute it from the export. Command Center carries it as a new campaign: $0 and 0 orders in its first 14 days. A ranking-lane raise to get a new campaign serving is legal inside the band; it stands, flagged.</t>
         </is>
       </c>
     </row>
@@ -9395,12 +9395,12 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>deploy</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
@@ -9410,7 +9410,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>A raise on a campaign the export does not carry: no status, child, or read to check it against. Confirm the campaign and its child first.</t>
+          <t>A raise on a campaign the export’s campaign list does not carry, so no reviewer can recompute it from the export. Command Center carries it as a new campaign: $0 and 0 orders in its first 14 days. A ranking-lane raise to get a new campaign serving is legal inside the band; it stands, flagged.</t>
         </is>
       </c>
     </row>
@@ -9460,12 +9460,12 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>deploy</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -9475,7 +9475,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>A raise on a campaign the export does not carry: no status, child, or read to check it against. Confirm the campaign and its child first.</t>
+          <t>A raise on a campaign the export’s campaign list does not carry, so no reviewer can recompute it from the export. Command Center carries it as a new campaign: $0 and 0 orders in its first 14 days. A ranking-lane raise to get a new campaign serving is legal inside the band; it stands, flagged.</t>
         </is>
       </c>
     </row>
@@ -9525,12 +9525,12 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>deploy</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -9540,7 +9540,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>A raise on a campaign the export does not carry: no status, child, or read to check it against. Confirm the campaign and its child first.</t>
+          <t>A raise on a campaign the export’s campaign list does not carry, so no reviewer can recompute it from the export. Command Center carries it as a new campaign: $0 and 0 orders in its first 14 days. A ranking-lane raise to get a new campaign serving is legal inside the band; it stands, flagged.</t>
         </is>
       </c>
     </row>
@@ -9590,12 +9590,12 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>deploy</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -9605,7 +9605,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>A raise on a campaign the export does not carry: no status, child, or read to check it against. Confirm the campaign and its child first.</t>
+          <t>A raise on a campaign the export’s campaign list does not carry, so no reviewer can recompute it from the export. Command Center carries it as a new campaign: $0 and 0 orders in its first 14 days. A ranking-lane raise to get a new campaign serving is legal inside the band; it stands, flagged.</t>
         </is>
       </c>
     </row>
@@ -9655,12 +9655,12 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>deploy</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>A raise on a campaign the export does not carry: no status, child, or read to check it against. Confirm the campaign and its child first.</t>
+          <t>A raise on a campaign the export’s campaign list does not carry, so no reviewer can recompute it from the export. Command Center carries it as a new campaign: $0 and 0 orders in its first 14 days. A ranking-lane raise to get a new campaign serving is legal inside the band; it stands, flagged.</t>
         </is>
       </c>
     </row>
@@ -9799,12 +9799,12 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>deploy</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>A raise on a campaign the export does not carry: no status, child, or read to check it against. Confirm the campaign and its child first.</t>
+          <t>A raise on a campaign the export’s campaign list does not carry, so no reviewer can recompute it from the export. Command Center carries it as a new campaign: $0 and 0 orders in its first 14 days. A ranking-lane raise to get a new campaign serving is legal inside the band; it stands, flagged.</t>
         </is>
       </c>
     </row>
@@ -10152,7 +10152,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 76 in FBA, 7 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 66 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
+          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 70 in FBA, 13 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 61 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -10170,7 +10170,7 @@
         <v>33</v>
       </c>
       <c r="R123" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S123" t="n">
         <v>0.5</v>
@@ -10179,7 +10179,7 @@
         <v>166</v>
       </c>
       <c r="U123" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="124">
@@ -10425,7 +10425,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 76 in FBA, 7 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 66 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
+          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 70 in FBA, 13 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 61 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -10443,7 +10443,7 @@
         <v>33</v>
       </c>
       <c r="R126" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S126" t="n">
         <v>0.5</v>
@@ -10452,7 +10452,7 @@
         <v>166</v>
       </c>
       <c r="U126" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="127">
@@ -10516,7 +10516,7 @@
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 76 in FBA, 7 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 66 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
+          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 70 in FBA, 13 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 61 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -10534,7 +10534,7 @@
         <v>33</v>
       </c>
       <c r="R127" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S127" t="n">
         <v>0.5</v>
@@ -10543,7 +10543,7 @@
         <v>166</v>
       </c>
       <c r="U127" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="128">
@@ -10880,7 +10880,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 76 in FBA, 7 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 66 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
+          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 70 in FBA, 13 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 61 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -10898,7 +10898,7 @@
         <v>33</v>
       </c>
       <c r="R131" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S131" t="n">
         <v>0.5</v>
@@ -10907,7 +10907,7 @@
         <v>166</v>
       </c>
       <c r="U131" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="132">
@@ -10971,7 +10971,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 76 in FBA, 7 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 66 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
+          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 70 in FBA, 13 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 61 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -10989,7 +10989,7 @@
         <v>33</v>
       </c>
       <c r="R132" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S132" t="n">
         <v>0.5</v>
@@ -10998,7 +10998,7 @@
         <v>166</v>
       </c>
       <c r="U132" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="133">
@@ -11153,7 +11153,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 76 in FBA, 7 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 66 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
+          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 70 in FBA, 13 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 61 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
@@ -11171,7 +11171,7 @@
         <v>33</v>
       </c>
       <c r="R134" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S134" t="n">
         <v>0.5</v>
@@ -11180,7 +11180,7 @@
         <v>166</v>
       </c>
       <c r="U134" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="135">
@@ -11881,7 +11881,7 @@
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 76 in FBA, 7 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 66 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
+          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 70 in FBA, 13 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 61 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
         </is>
       </c>
       <c r="N142" t="inlineStr">
@@ -11899,7 +11899,7 @@
         <v>33</v>
       </c>
       <c r="R142" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S142" t="n">
         <v>0.5</v>
@@ -11908,7 +11908,7 @@
         <v>166</v>
       </c>
       <c r="U142" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="143">
@@ -11972,7 +11972,7 @@
       </c>
       <c r="M143" t="inlineStr">
         <is>
-          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 76 in FBA, 7 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 66 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
+          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 70 in FBA, 13 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 61 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
         </is>
       </c>
       <c r="N143" t="inlineStr">
@@ -11990,7 +11990,7 @@
         <v>33</v>
       </c>
       <c r="R143" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S143" t="n">
         <v>0.5</v>
@@ -11999,7 +11999,7 @@
         <v>166</v>
       </c>
       <c r="U143" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="144">
@@ -12518,7 +12518,7 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 76 in FBA, 7 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 66 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
+          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 70 in FBA, 13 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 61 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
@@ -12536,7 +12536,7 @@
         <v>33</v>
       </c>
       <c r="R149" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S149" t="n">
         <v>0.5</v>
@@ -12545,7 +12545,7 @@
         <v>166</v>
       </c>
       <c r="U149" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="150">
@@ -13610,7 +13610,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 76 in FBA, 7 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 66 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
+          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 70 in FBA, 13 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 61 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -13628,7 +13628,7 @@
         <v>33</v>
       </c>
       <c r="R161" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S161" t="n">
         <v>0.5</v>
@@ -13637,7 +13637,7 @@
         <v>166</v>
       </c>
       <c r="U161" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="162">
@@ -13701,7 +13701,7 @@
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 76 in FBA, 7 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 66 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
+          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 70 in FBA, 13 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 61 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
@@ -13719,7 +13719,7 @@
         <v>33</v>
       </c>
       <c r="R162" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S162" t="n">
         <v>0.5</v>
@@ -13728,7 +13728,7 @@
         <v>166</v>
       </c>
       <c r="U162" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="163">
@@ -15521,7 +15521,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 76 in FBA, 7 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 66 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
+          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 70 in FBA, 13 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 61 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -15539,7 +15539,7 @@
         <v>33</v>
       </c>
       <c r="R182" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S182" t="n">
         <v>0.5</v>
@@ -15548,7 +15548,7 @@
         <v>166</v>
       </c>
       <c r="U182" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="183">
@@ -15794,7 +15794,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 76 in FBA, 7 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 66 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
+          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 70 in FBA, 13 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 61 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -15812,7 +15812,7 @@
         <v>33</v>
       </c>
       <c r="R185" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S185" t="n">
         <v>0.5</v>
@@ -15821,7 +15821,7 @@
         <v>166</v>
       </c>
       <c r="U185" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="186">
@@ -20799,7 +20799,7 @@
       </c>
       <c r="M240" t="inlineStr">
         <is>
-          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 76 in FBA, 7 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 66 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
+          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 70 in FBA, 13 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 61 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
         </is>
       </c>
       <c r="N240" t="inlineStr">
@@ -20817,7 +20817,7 @@
         <v>33</v>
       </c>
       <c r="R240" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S240" t="n">
         <v>0.5</v>
@@ -20826,7 +20826,7 @@
         <v>166</v>
       </c>
       <c r="U240" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="241">
@@ -21072,7 +21072,7 @@
       </c>
       <c r="M243" t="inlineStr">
         <is>
-          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 76 in FBA, 7 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 66 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
+          <t>Due under the push. At today’s pace the planner gives the hero 33 days, but this run pushes Cal King, and at the push pace the run reads about 21 days. Its 120 inbound units have no date and the next PO is 5 November. Source BAMBOO-CALIFKING-WHITE: 49 in FBA, 3 reserved, 120 inbound, 1.62/day, 33 days left. Target BAMBOO-CALIFKING-OLIVE: 70 in FBA, 13 reserved, 30 inbound, 0.50/day, 166 days left. The 15 campaign(s) making this move carry 0.6 ad orders a day, which leaves the target about 61 days of cover. Watch the conversion rate: Olive sells 0.5 a day against White’s 1.6, and the push now ranks on it.</t>
         </is>
       </c>
       <c r="N243" t="inlineStr">
@@ -21090,7 +21090,7 @@
         <v>33</v>
       </c>
       <c r="R243" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="S243" t="n">
         <v>0.5</v>
@@ -21099,7 +21099,7 @@
         <v>166</v>
       </c>
       <c r="U243" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="244">
@@ -23448,12 +23448,12 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>deploy</t>
         </is>
       </c>
       <c r="L274" t="inlineStr">
@@ -23463,7 +23463,7 @@
       </c>
       <c r="M274" t="inlineStr">
         <is>
-          <t>A raise on a campaign the export does not carry: no status, child, or read to check it against. Confirm the campaign and its child first.</t>
+          <t>A raise on a campaign the export’s campaign list does not carry, so no reviewer can recompute it from the export. Command Center carries it as a new campaign: $0 and 0 orders in its first 14 days. A ranking-lane raise to get a new campaign serving is legal inside the band; it stands, flagged.</t>
         </is>
       </c>
     </row>
@@ -23513,12 +23513,12 @@
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>deploy</t>
         </is>
       </c>
       <c r="L275" t="inlineStr">
@@ -23528,7 +23528,7 @@
       </c>
       <c r="M275" t="inlineStr">
         <is>
-          <t>A raise on a campaign the export does not carry: no status, child, or read to check it against. Confirm the campaign and its child first.</t>
+          <t>A raise on a campaign the export’s campaign list does not carry, so no reviewer can recompute it from the export. Command Center carries it as a new campaign: $0 and 0 orders in its first 14 days. A ranking-lane raise to get a new campaign serving is legal inside the band; it stands, flagged.</t>
         </is>
       </c>
     </row>
@@ -23578,12 +23578,12 @@
       </c>
       <c r="J276" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>deploy</t>
         </is>
       </c>
       <c r="L276" t="inlineStr">
@@ -23593,7 +23593,7 @@
       </c>
       <c r="M276" t="inlineStr">
         <is>
-          <t>A raise on a campaign the export does not carry: no status, child, or read to check it against. Confirm the campaign and its child first.</t>
+          <t>A raise on a campaign the export’s campaign list does not carry, so no reviewer can recompute it from the export. Command Center carries it as a new campaign: $0 and 0 orders in its first 14 days. A ranking-lane raise to get a new campaign serving is legal inside the band; it stands, flagged.</t>
         </is>
       </c>
     </row>
@@ -23959,12 +23959,12 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>deploy</t>
         </is>
       </c>
       <c r="L281" t="inlineStr">
@@ -23974,7 +23974,7 @@
       </c>
       <c r="M281" t="inlineStr">
         <is>
-          <t>A raise on a campaign the export does not carry: no status, child, or read to check it against. Confirm the campaign and its child first.</t>
+          <t>A raise on a campaign the export’s campaign list does not carry, so no reviewer can recompute it from the export. Command Center carries it as a new campaign: $0 and 0 orders in its first 14 days. A ranking-lane raise to get a new campaign serving is legal inside the band; it stands, flagged.</t>
         </is>
       </c>
     </row>
@@ -24103,12 +24103,12 @@
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>deploy</t>
         </is>
       </c>
       <c r="L283" t="inlineStr">
@@ -24118,7 +24118,7 @@
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>A raise on a campaign the export does not carry: no status, child, or read to check it against. Confirm the campaign and its child first.</t>
+          <t>A raise on a campaign the export’s campaign list does not carry, so no reviewer can recompute it from the export. Command Center carries it as a new campaign: $0 and 0 orders in its first 14 days. A ranking-lane raise to get a new campaign serving is legal inside the band; it stands, flagged.</t>
         </is>
       </c>
     </row>
@@ -24168,12 +24168,12 @@
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>deploy</t>
         </is>
       </c>
       <c r="L284" t="inlineStr">
@@ -24183,7 +24183,7 @@
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>A raise on a campaign the export does not carry: no status, child, or read to check it against. Confirm the campaign and its child first.</t>
+          <t>A raise on a campaign the export’s campaign list does not carry, so no reviewer can recompute it from the export. Command Center carries it as a new campaign: $0 and 0 orders in its first 14 days. A ranking-lane raise to get a new campaign serving is legal inside the band; it stands, flagged.</t>
         </is>
       </c>
     </row>
@@ -34472,10 +34472,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="E4" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F4" t="n">
         <v>30</v>
@@ -34484,7 +34484,7 @@
         <v>0.3</v>
       </c>
       <c r="H4" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -34492,7 +34492,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -34691,7 +34691,7 @@
         <v>11</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
         <v>48</v>
@@ -34700,7 +34700,7 @@
         <v>1.16</v>
       </c>
       <c r="H8" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -34708,7 +34708,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -34799,7 +34799,7 @@
         <v>14</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F10" t="n">
         <v>60</v>
@@ -34808,7 +34808,7 @@
         <v>0.41</v>
       </c>
       <c r="H10" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -34816,7 +34816,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -34958,10 +34958,10 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E13" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F13" t="n">
         <v>30</v>
@@ -35012,7 +35012,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E14" t="n">
         <v>1</v>
@@ -35024,7 +35024,7 @@
         <v>0.34</v>
       </c>
       <c r="H14" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -35032,7 +35032,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -35120,10 +35120,10 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
         <v>60</v>
@@ -37010,7 +37010,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E51" t="n">
         <v>7</v>
@@ -37022,7 +37022,7 @@
         <v>0.89</v>
       </c>
       <c r="H51" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -37030,7 +37030,7 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -37226,10 +37226,10 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E55" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F55" t="n">
         <v>60</v>
@@ -37496,7 +37496,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E60" t="n">
         <v>8</v>
@@ -37508,7 +37508,7 @@
         <v>0.73</v>
       </c>
       <c r="H60" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
@@ -37516,7 +37516,7 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
@@ -37604,7 +37604,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E62" t="n">
         <v>3</v>
@@ -37616,7 +37616,7 @@
         <v>1.22</v>
       </c>
       <c r="H62" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
@@ -37624,7 +37624,7 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -37877,7 +37877,7 @@
         <v>17</v>
       </c>
       <c r="E67" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F67" t="n">
         <v>30</v>
@@ -37886,7 +37886,7 @@
         <v>0.58</v>
       </c>
       <c r="H67" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
@@ -37894,7 +37894,7 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -38877,11 +38877,11 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>BAMBOO-CALIFKING-OLIVE: 76 in FBA, 7 reserved, 30 inbound, 0.50/day, 166 days left</t>
+          <t>BAMBOO-CALIFKING-OLIVE: 70 in FBA, 13 reserved, 30 inbound, 0.50/day, 166 days left</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="I3" t="n">
         <v>15</v>
@@ -39379,7 +39379,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Re-point by hand to BAMBOO-FULL-OLIVE: 101 in FBA, 3 reserved, 1.22/day, 86 days left.</t>
+          <t>Re-point by hand to BAMBOO-FULL-OLIVE: 100 in FBA, 3 reserved, 1.22/day, 85 days left.</t>
         </is>
       </c>
     </row>
@@ -39455,7 +39455,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Re-point by hand to BAMBOO-CALIFKING-TAUPE: 49 in FBA, 2 reserved, 60 inbound, 2.07/day, 25 days left.</t>
+          <t>Re-point by hand to BAMBOO-CALIFKING-TAUPE: 50 in FBA, 1 reserved, 60 inbound, 2.07/day, 25 days left.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add SCS4 audit review for run 20260924-7aed7be1; fix rename check
SCS4 (Sleephoria Cooling Sheets 4 Piece): review docx and per-row
workbook, judged on the Sellerboard planner for all 63 children.
Weekly sales fell 45% in three weeks, so the run's TACoS is priced on a
stale base; 31 King campaigns must leave King Graphite (15 days); the
Twin swaps onto Twin White (12 units) are held; one of four freezes is
a real loss.

The rename check read only SATIN SKUs, so the bamboo reviews held no
renames. It now reads every planner SKU. DBS4, DBS6 and DSS6 are
re-issued with the corrected rename rows. The method doc gains the
size-fix exception and the undated-inbound rule.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECNUyLvUafHehET6NevFNz
</commit_message>
<xml_diff>
--- a/docs/reviews/DBS4_Review_Rows_20260924-5e8a0f10.xlsx
+++ b/docs/reviews/DBS4_Review_Rows_20260924-5e8a0f10.xlsx
@@ -30366,17 +30366,17 @@
       </c>
       <c r="K367" t="inlineStr">
         <is>
-          <t>deploy</t>
+          <t>after the swap</t>
         </is>
       </c>
       <c r="L367" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="M367" t="inlineStr">
         <is>
-          <t>Naming only.</t>
+          <t>Stamps BAMBOO-QUEEN-OLIVE, the target of a swap that is due on stock (at risk on the source). Rename once the swap is done by hand, not before.</t>
         </is>
       </c>
       <c r="N367" t="inlineStr">
@@ -30682,17 +30682,17 @@
       </c>
       <c r="K371" t="inlineStr">
         <is>
-          <t>deploy</t>
+          <t>after the swap</t>
         </is>
       </c>
       <c r="L371" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="M371" t="inlineStr">
         <is>
-          <t>Naming only.</t>
+          <t>Stamps BAMBOO-QUEEN-OLIVE, the target of a swap that is due on stock (at risk on the source). Rename once the swap is done by hand, not before.</t>
         </is>
       </c>
       <c r="N371" t="inlineStr">
@@ -31625,22 +31625,22 @@
       </c>
       <c r="J383" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>hold</t>
         </is>
       </c>
       <c r="K383" t="inlineStr">
         <is>
-          <t>deploy</t>
+          <t>hold</t>
         </is>
       </c>
       <c r="L383" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="M383" t="inlineStr">
         <is>
-          <t>Naming only.</t>
+          <t>The name stamps BAMBOO-KING-LIGHTBLUE: 403 in FBA, 51 reserved, 4.13/day, 110 days left, but the ad serves BAMBOO-KING-WHITE: 204 in FBA, 106 reserved, 2430 inbound, 9.81/day, 32 days left, and the swap cannot load (and the swap itself is held on stock). The name would describe a child the campaign does not advertise.</t>
         </is>
       </c>
       <c r="N383" t="inlineStr">

</xml_diff>